<commit_message>
part 1 - Final version
</commit_message>
<xml_diff>
--- a/Output_2026/SAAM_Part1_EUR_results.xlsx
+++ b/Output_2026/SAAM_Part1_EUR_results.xlsx
@@ -427,17 +427,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Ann. Return Arith. (%)</t>
+          <t>Ann Ret Arith (%)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Ann. Return Geom. (%)</t>
+          <t>Ann Ret Geom (%)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Ann. Vol (%)</t>
+          <t>Ann Vol (%)</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
@@ -447,12 +447,12 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Min Mo. (%)</t>
+          <t>Min Mo (%)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Max Mo. (%)</t>
+          <t>Max Mo (%)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
@@ -464,7 +464,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Val-Wgt P^(vw)</t>
+          <t>Value-Weighted</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -492,7 +492,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Min-Var P_oos^(mv)</t>
+          <t>Min-Variance</t>
         </is>
       </c>
       <c r="B3" t="n">

</xml_diff>